<commit_message>
Scope Studio 7 to LO 7-1 through 7-7
The studio no longer practises PERT. Part 4 now totals the register's
contingency reserve, asks who controls each reserve, and places one time
buffer in the Week 6 network using the chapter's four placement rules. The
workbook's PERT sheet is replaced by a Reserve and buffer sheet that reads
the register's total. The Thursday title drops its schedule half in the
lab, the week page's front matter and meta block, and the deck's closing
slides, so all four agree. PERT stays in Tuesday's session and the appendix
exercises.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/files/week-07-risk-studio.xlsx
+++ b/files/week-07-risk-studio.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Register" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scales" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matrix" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERT" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Register" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Scales" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Matrix" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Reserve and buffer" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reconciliation" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,9 +20,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -85,7 +84,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -107,55 +106,11 @@
         <color rgb="00D9D9D9"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00D9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00D9D9D9"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D9D9D9"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D9D9D9"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -189,14 +144,8 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1712,446 +1661,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PERT · revised three-point estimates (workdays)</t>
+          <t>Reserve and buffer · LO 7-7</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>These estimates replace the ones in the notes. Enter your own formulas in the yellow cells.</t>
+          <t>The reserve total comes from the Register. Fill the yellow cells; the budget lines calculate.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Activity</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Predecessors</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>b</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>t_e</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Variance</t>
-        </is>
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Baseline budget (from the notes)</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>70000</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="B5" s="15" t="inlineStr">
-        <is>
-          <t>Event brief</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F5" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Contingency reserve (total of the Register's Reserve column)</t>
+        </is>
+      </c>
+      <c r="B5" s="15">
+        <f>Register!Q13</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="B6" s="15" t="inlineStr">
-        <is>
-          <t>Venue</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="6" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="G6" s="16" t="n"/>
-      <c r="H6" s="16" t="n"/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Project budget (baseline + contingency reserve)</t>
+        </is>
+      </c>
+      <c r="B6" s="15">
+        <f>B4+B5</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="B7" s="15" t="inlineStr">
-        <is>
-          <t>Program draft</t>
-        </is>
-      </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B8" s="15" t="inlineStr">
-        <is>
-          <t>Registration</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E8" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F8" s="6" t="n">
-        <v>13</v>
-      </c>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Reserve as a share of baseline</t>
+        </is>
+      </c>
+      <c r="B7" s="16">
+        <f>IF(B4&gt;0,B5/B4,"")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>Speakers</t>
-        </is>
-      </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>16</v>
-      </c>
-      <c r="G9" s="16" t="n"/>
-      <c r="H9" s="16" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="B10" s="15" t="inlineStr">
-        <is>
-          <t>Exhibitors</t>
-        </is>
-      </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E10" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="F10" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="16" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="B11" s="15" t="inlineStr">
-        <is>
-          <t>Publish program</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>D, E</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>9</v>
-      </c>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="B12" s="15" t="inlineStr">
-        <is>
-          <t>Materials</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>F, G</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E12" s="6" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" s="6" t="n">
-        <v>6</v>
-      </c>
-      <c r="G12" s="16" t="n"/>
-      <c r="H12" s="16" t="n"/>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Who controls it, and what it pays for</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Contingency reserve</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Management reserve</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
-        <is>
-          <t>Rehearsal</t>
-        </is>
-      </c>
-      <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="E13" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="G13" s="16" t="n"/>
-      <c r="H13" s="16" t="n"/>
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>One time buffer in the Week 6 conference network</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Activity (ID and name)</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Placement rule</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Paths</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Path</t>
-        </is>
-      </c>
-      <c r="B17" s="17" t="n"/>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="3" t="inlineStr">
-        <is>
-          <t>Sum t_e</t>
-        </is>
-      </c>
-      <c r="E17" s="3" t="inlineStr">
-        <is>
-          <t>Sum variance</t>
-        </is>
-      </c>
-      <c r="F17" s="3" t="inlineStr">
-        <is>
-          <t>σ</t>
-        </is>
-      </c>
-      <c r="G17" s="3" t="inlineStr">
-        <is>
-          <t>Z at T_S</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>P(finish ≤ T_S)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>A–B–D–G–H–I</t>
-        </is>
-      </c>
-      <c r="D18" s="16" t="n"/>
-      <c r="E18" s="16" t="n"/>
-      <c r="F18" s="16" t="n"/>
-      <c r="G18" s="16" t="n"/>
-      <c r="H18" s="19" t="n"/>
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Days held</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Reason (one or two sentences)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>A–C–E–G–H–I</t>
-        </is>
-      </c>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="16" t="n"/>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="19" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>A–C–F–H–I</t>
-        </is>
-      </c>
-      <c r="D20" s="16" t="n"/>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="16" t="n"/>
-      <c r="G20" s="16" t="n"/>
-      <c r="H20" s="19" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
-        <is>
-          <t>Scheduled time T_S (sponsor's date)</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
-        <is>
-          <t>Z for 90% confidence</t>
-        </is>
-      </c>
-      <c r="D23" t="n">
-        <v>1.2816</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="8" t="inlineStr">
-        <is>
-          <t>T_E + 1.28σ on the critical path</t>
-        </is>
-      </c>
-      <c r="D24" s="20" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Tip: =NORM.S.DIST(Z, TRUE) returns the probability for a Z value.</t>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>If the reserve is more than a quarter of the baseline, say which rows drive it and whether that is judgement or padding.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A19:C19"/>
-  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation sqref="B15" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"After an activity with severe risk,At a merge activity,On a noncritical path with little slack,Before an activity that needs a scarce resource"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" error="Whole days, 0 to 30." type="whole" operator="between">
+      <formula1>0</formula1>
+      <formula2>30</formula2>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2214,7 +1866,7 @@
       </c>
     </row>
     <row r="5" ht="48" customHeight="1">
-      <c r="A5" s="21" t="n">
+      <c r="A5" s="17" t="n">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -2223,7 +1875,7 @@
       <c r="E5" s="5" t="n"/>
     </row>
     <row r="6" ht="48" customHeight="1">
-      <c r="A6" s="21" t="n">
+      <c r="A6" s="17" t="n">
         <v>2</v>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -2232,7 +1884,7 @@
       <c r="E6" s="5" t="n"/>
     </row>
     <row r="7" ht="48" customHeight="1">
-      <c r="A7" s="21" t="n">
+      <c r="A7" s="17" t="n">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="n"/>
@@ -2241,7 +1893,7 @@
       <c r="E7" s="5" t="n"/>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="21" t="n">
+      <c r="A8" s="17" t="n">
         <v>4</v>
       </c>
       <c r="B8" s="5" t="n"/>
@@ -2250,7 +1902,7 @@
       <c r="E8" s="5" t="n"/>
     </row>
     <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="17" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="n"/>
@@ -2259,7 +1911,7 @@
       <c r="E9" s="5" t="n"/>
     </row>
     <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="21" t="n">
+      <c r="A10" s="17" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="5" t="n"/>
@@ -2268,7 +1920,7 @@
       <c r="E10" s="5" t="n"/>
     </row>
     <row r="11" ht="48" customHeight="1">
-      <c r="A11" s="21" t="n">
+      <c r="A11" s="17" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="5" t="n"/>
@@ -2277,7 +1929,7 @@
       <c r="E11" s="5" t="n"/>
     </row>
     <row r="12" ht="48" customHeight="1">
-      <c r="A12" s="21" t="n">
+      <c r="A12" s="17" t="n">
         <v>8</v>
       </c>
       <c r="B12" s="5" t="n"/>
@@ -2286,7 +1938,7 @@
       <c r="E12" s="5" t="n"/>
     </row>
     <row r="13" ht="48" customHeight="1">
-      <c r="A13" s="21" t="n">
+      <c r="A13" s="17" t="n">
         <v>9</v>
       </c>
       <c r="B13" s="5" t="n"/>
@@ -2295,7 +1947,7 @@
       <c r="E13" s="5" t="n"/>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="21" t="n">
+      <c r="A14" s="17" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="5" t="n"/>

</xml_diff>